<commit_message>
sprint7, ganttChart, burndownChart scrumBoard update (little correction in sprint4)
</commit_message>
<xml_diff>
--- a/SE202526/Management/Sprint4/GanttSprint4.xlsx
+++ b/SE202526/Management/Sprint4/GanttSprint4.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr filterPrivacy="1" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B13BA68-A8C7-4AEA-BEC8-3F02E6522646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B4AC672-A537-404B-A156-E60FB7AE55C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1388,19 +1388,19 @@
         <v>26</v>
       </c>
       <c r="D5" s="7">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="E5" s="7">
         <v>5</v>
       </c>
       <c r="F5" s="7">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="G5" s="7">
         <v>4</v>
       </c>
       <c r="H5" s="4">
-        <v>0.25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="2:68" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1411,13 +1411,13 @@
         <v>27</v>
       </c>
       <c r="D6" s="7">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="E6" s="7">
         <v>7</v>
       </c>
       <c r="F6" s="7">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="G6" s="7">
         <v>3</v>
@@ -1434,19 +1434,19 @@
         <v>28</v>
       </c>
       <c r="D7" s="7">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="E7" s="7">
         <v>7</v>
       </c>
       <c r="F7" s="7">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="G7" s="7">
         <v>3</v>
       </c>
       <c r="H7" s="4">
-        <v>0.35</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="2:68" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1457,19 +1457,19 @@
         <v>29</v>
       </c>
       <c r="D8" s="7">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="E8" s="7">
         <v>7</v>
       </c>
       <c r="F8" s="7">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="G8" s="7">
         <v>2</v>
       </c>
       <c r="H8" s="4">
-        <v>0.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="2:68" ht="30" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>